<commit_message>
xlsx: exclude Excel Table Total Row from data range and banding
RegisterTable treated a table's totalsRowCount rows as ordinary data
rows, so a real totals-row formula like
=SUBTOTAL(109,Table1[Column]) would structurally include its own
cell in the aggregate it computes. ApplyTableBanding had the same
gap visually (banding the totals row like a data row).

Both now read totalsRowCount from <table> and exclude that many
rows from the bottom of the range. Per-column totalsRowFunction/
totalsRowLabel are still not read at all -- nothing in this app
would consume them (no live Total Row UI), and the totals row's own
formula already calculates correctly through the normal per-cell
pipeline once its range is right.

tests/sample_table.xlsx gained a real totals row to cover this; also
fixed an unrelated changelog entry accidentally split across two
bullets in a previous commit.
</commit_message>
<xml_diff>
--- a/translators/xlsx/tests/sample_table.xlsx
+++ b/translators/xlsx/tests/sample_table.xlsx
@@ -42,11 +42,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabella1" displayName="Tabella1" ref="A1:B4" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabella1" displayName="Tabella1" ref="A1:B5" totalsRowCount="1">
   <autoFilter ref="A1:B4"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Codice"/>
-    <tableColumn id="2" name="Descrizione"/>
+    <tableColumn id="2" name="Descrizione" totalsRowFunction="count"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -103,6 +103,18 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>